<commit_message>
2023-05-30 Lambda bug 修复
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-wms/src/main/resources/excel/soOutstock.xlsx
+++ b/erp-server/erp-server-wms/src/main/resources/excel/soOutstock.xlsx
@@ -110,6 +110,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="宋体"/>
+        <family val="3"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
@@ -141,6 +142,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="宋体"/>
+        <family val="3"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
@@ -176,6 +178,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="宋体"/>
+        <family val="3"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
@@ -184,14 +187,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>发货组织</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.deliveryOrgName}</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t>销售组织</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -231,6 +226,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="宋体"/>
+        <family val="3"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
@@ -266,6 +262,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="宋体"/>
+        <family val="3"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
@@ -297,6 +294,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="宋体"/>
+        <family val="3"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
@@ -313,11 +311,20 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="宋体"/>
+        <family val="3"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
       <t>}</t>
     </r>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>库存组织</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.warehouseOrgName}</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -326,7 +333,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="178" formatCode="yyyy/m/d;@"/>
+    <numFmt numFmtId="176" formatCode="yyyy/m/d;@"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -438,7 +445,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -757,10 +764,10 @@
         <v>28</v>
       </c>
       <c r="H1" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="I1" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>32</v>
       </c>
       <c r="J1" s="5" t="s">
         <v>2</v>
@@ -769,19 +776,19 @@
         <v>3</v>
       </c>
       <c r="L1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="N1" s="4" t="s">
-        <v>38</v>
-      </c>
       <c r="O1" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>41</v>
       </c>
       <c r="Q1" s="5" t="s">
         <v>4</v>
@@ -825,10 +832,10 @@
         <v>29</v>
       </c>
       <c r="H2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>33</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>13</v>
@@ -837,22 +844,22 @@
         <v>14</v>
       </c>
       <c r="L2" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="M2" s="4" t="s">
         <v>35</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>37</v>
       </c>
       <c r="N2" s="7" t="s">
         <v>15</v>
       </c>
       <c r="O2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="P2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="P2" s="4" t="s">
-        <v>42</v>
-      </c>
       <c r="Q2" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="R2" s="5" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
2023-05-31 Lambda bug 修复
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-wms/src/main/resources/excel/soOutstock.xlsx
+++ b/erp-server/erp-server-wms/src/main/resources/excel/soOutstock.xlsx
@@ -123,6 +123,14 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
+    <t>作废状态</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>客户</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
     <r>
       <t>{.</t>
     </r>
@@ -135,7 +143,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>typeName</t>
+      <t>customerName</t>
     </r>
     <r>
       <rPr>
@@ -151,11 +159,23 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>作废状态</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>客户</t>
+    <t>销售组织</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.salesOrgName}</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>应发数量</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.planQty}</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>实发数量</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
@@ -171,7 +191,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>customerName</t>
+      <t>actualQty</t>
     </r>
     <r>
       <rPr>
@@ -187,23 +207,11 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>销售组织</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.salesOrgName}</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>应发数量</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.planQty}</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>实发数量</t>
+    <t>库存单位</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>出货仓库</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
@@ -219,7 +227,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>actualQty</t>
+      <t>warehouseName</t>
     </r>
     <r>
       <rPr>
@@ -235,11 +243,7 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>库存单位</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>出货仓库</t>
+    <t>出库日期</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
@@ -255,7 +259,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>warehouseName</t>
+      <t>actualDeliveryDate</t>
     </r>
     <r>
       <rPr>
@@ -271,23 +275,8 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>出库日期</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>{.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>actualDeliveryDate</t>
+    <r>
+      <t>{.planDeliveryDate</t>
     </r>
     <r>
       <rPr>
@@ -303,28 +292,15 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <t>{.planDeliveryDate</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>}</t>
-    </r>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t>库存组织</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
     <t>{.warehouseOrgName}</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.orderTypeName}</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -758,16 +734,16 @@
         <v>1</v>
       </c>
       <c r="F1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>28</v>
-      </c>
       <c r="H1" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J1" s="5" t="s">
         <v>2</v>
@@ -776,19 +752,19 @@
         <v>3</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="N1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="O1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="O1" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="P1" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="Q1" s="5" t="s">
         <v>4</v>
@@ -820,7 +796,7 @@
         <v>24</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>11</v>
@@ -829,13 +805,13 @@
         <v>12</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>13</v>
@@ -844,22 +820,22 @@
         <v>14</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="N2" s="7" t="s">
         <v>15</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>41</v>
       </c>
       <c r="R2" s="5" t="s">
         <v>16</v>

</xml_diff>